<commit_message>
feat: agregar script ejecutable .bat para pipeline autonomo e indices de optimizacion SQL
</commit_message>
<xml_diff>
--- a/Reporte_Ventas_Limpio.xlsx
+++ b/Reporte_Ventas_Limpio.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,52 +421,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID Cliente</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Nombre Cliente</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ID Producto</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Nombre Producto</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fecha Venta</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Total Cantidad Vendida</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Total Ingresos</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Ticket Promedio Por Producto</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Comentarios_Cliente</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Descuento_Aplicado</t>
         </is>
@@ -501,7 +489,7 @@
           <t>Laptop Pro 15</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="1" t="n">
         <v>46318.54833159722</v>
       </c>
       <c r="F2" t="n">
@@ -539,7 +527,7 @@
           <t>Laptop Pro 15</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>46319.39726443287</v>
       </c>
       <c r="F3" t="n">
@@ -577,7 +565,7 @@
           <t>Laptop Pro 15</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="1" t="n">
         <v>46321.69777728009</v>
       </c>
       <c r="F4" t="n">
@@ -615,7 +603,7 @@
           <t>Laptop Pro 15</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>46321.71759525463</v>
       </c>
       <c r="F5" t="n">
@@ -653,7 +641,7 @@
           <t>Cargador Carga Rápida</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>46319.39726450232</v>
       </c>
       <c r="F6" t="n">
@@ -691,7 +679,7 @@
           <t>Cargador Carga Rápida</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>46321.69777734954</v>
       </c>
       <c r="F7" t="n">
@@ -729,7 +717,7 @@
           <t>Cargador Carga Rápida</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>46321.71759528935</v>
       </c>
       <c r="F8" t="n">
@@ -767,7 +755,7 @@
           <t>Laptop Pro 15</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>46319.39726450232</v>
       </c>
       <c r="F9" t="n">
@@ -805,7 +793,7 @@
           <t>Laptop Pro 15</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>46321.69777734954</v>
       </c>
       <c r="F10" t="n">
@@ -843,7 +831,7 @@
           <t>Laptop Pro 15</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="1" t="n">
         <v>46321.71759528935</v>
       </c>
       <c r="F11" t="n">
@@ -881,7 +869,7 @@
           <t>Teclado Mecánico RGB</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="1" t="n">
         <v>46319.3972644676</v>
       </c>
       <c r="F12" t="n">
@@ -919,7 +907,7 @@
           <t>Teclado Mecánico RGB</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46321.69777731482</v>
       </c>
       <c r="F13" t="n">
@@ -957,7 +945,7 @@
           <t>Teclado Mecánico RGB</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="1" t="n">
         <v>46321.71759525463</v>
       </c>
       <c r="F14" t="n">
@@ -995,7 +983,7 @@
           <t>Audífonos HyperX</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46319.3972644676</v>
       </c>
       <c r="F15" t="n">
@@ -1033,7 +1021,7 @@
           <t>Audífonos HyperX</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="1" t="n">
         <v>46321.69777731482</v>
       </c>
       <c r="F16" t="n">
@@ -1071,7 +1059,7 @@
           <t>Audífonos HyperX</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="1" t="n">
         <v>46321.71759525463</v>
       </c>
       <c r="F17" t="n">
@@ -1109,7 +1097,7 @@
           <t>Silla Ergonómica Pro</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46319.3972644676</v>
       </c>
       <c r="F18" t="n">
@@ -1147,7 +1135,7 @@
           <t>Silla Ergonómica Pro</t>
         </is>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="1" t="n">
         <v>46321.69777731482</v>
       </c>
       <c r="F19" t="n">
@@ -1185,7 +1173,7 @@
           <t>Silla Ergonómica Pro</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>46321.71759528935</v>
       </c>
       <c r="F20" t="n">

</xml_diff>